<commit_message>
docs(week1): lock appendix G product decisions
</commit_message>
<xml_diff>
--- a/docs/week1/05_本周验收台账.xlsx
+++ b/docs/week1/05_本周验收台账.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A验收" sheetId="1" r:id="R5e96ee7b7d8d4ef9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B验收" sheetId="2" r:id="Rd7e6fa04ec7d4c33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C验收" sheetId="3" r:id="Raeab5ad31af342bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="协作交接" sheetId="4" r:id="R32d0eeb9d36d4585"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20样本评测" sheetId="5" r:id="R9068e0fac1b74fd7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="6" r:id="R28ef797d9bd941e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="7" r:id="Raf9a775e48104b6f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="A验收" sheetId="1" r:id="R06c5351843914d8f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B验收" sheetId="2" r:id="R3f1c12d3f4a04a9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="C验收" sheetId="3" r:id="R531fce16b9d84f3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="协作交接" sheetId="4" r:id="R97e17551ab3b4fab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20样本评测" sheetId="5" r:id="Rb4404f0fc14140fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="证据索引" sheetId="6" r:id="R8eeb60cda057480f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="7" r:id="Ra92654e4e34a4a36"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -204,7 +204,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -215,7 +215,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -226,7 +226,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -237,7 +237,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -248,7 +248,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -259,7 +259,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -270,7 +270,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -281,7 +281,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -292,7 +292,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -303,7 +303,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -314,7 +314,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -325,7 +325,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -335,7 +335,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -345,7 +345,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -356,7 +356,7 @@
         <x:color rgb="FF375623"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE2F0D9"/>
         </x:patternFill>
       </x:fill>
@@ -367,7 +367,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -5784,7 +5784,7 @@
         <x:v>公开响应敏感字段命中</x:v>
       </x:c>
       <x:c r="D19" s="12" t="str">
-        <x:v>姓名、private_ref、Cookie、密钥、堆栈为0</x:v>
+        <x:v>姓名、头像、二维码、联系方式、会议入口、private_ref、Cookie、密钥、堆栈为0</x:v>
       </x:c>
       <x:c r="E19" s="18" t="str">
         <x:v>数值</x:v>
@@ -5924,7 +5924,7 @@
       <x:c r="AA21" s="27"/>
       <x:c r="AB21" s="27"/>
     </x:row>
-    <x:row r="22" ht="33" customHeight="1">
+    <x:row r="22" ht="24" hidden="0" customHeight="1">
       <x:c r="A22" s="18" t="str">
         <x:v>C-17</x:v>
       </x:c>
@@ -5932,10 +5932,10 @@
         <x:v>46285.99930555555</x:v>
       </x:c>
       <x:c r="C22" s="12" t="str">
-        <x:v>公共HTTPS测试URL</x:v>
+        <x:v>React/Vite前端迁移</x:v>
       </x:c>
       <x:c r="D22" s="12" t="str">
-        <x:v>公网可打开首页并完成传统检索</x:v>
+        <x:v>React+TypeScript+Vite消费Flask API，首页与传统检索可运行</x:v>
       </x:c>
       <x:c r="E22" s="18" t="str">
         <x:v>是非</x:v>
@@ -5973,7 +5973,7 @@
       <x:c r="AA22" s="27"/>
       <x:c r="AB22" s="27"/>
     </x:row>
-    <x:row r="23" ht="33" customHeight="1">
+    <x:row r="23" ht="36" hidden="0" customHeight="1">
       <x:c r="A23" s="18" t="str">
         <x:v>C-18</x:v>
       </x:c>
@@ -5981,10 +5981,10 @@
         <x:v>46285.99930555555</x:v>
       </x:c>
       <x:c r="C23" s="12" t="str">
-        <x:v>健康检查</x:v>
+        <x:v>健康检查与云端部署清单</x:v>
       </x:c>
       <x:c r="D23" s="12" t="str">
-        <x:v>公共GET /healthz返回2xx并报告组件状态</x:v>
+        <x:v>LAN GET /healthz返回2xx；服务器、域名、反向代理、证书和续期清单齐全</x:v>
       </x:c>
       <x:c r="E23" s="18" t="str">
         <x:v>是非</x:v>
@@ -6022,7 +6022,7 @@
       <x:c r="AA23" s="27"/>
       <x:c r="AB23" s="27"/>
     </x:row>
-    <x:row r="24" ht="33" customHeight="1">
+    <x:row r="24" ht="36" hidden="0" customHeight="1">
       <x:c r="A24" s="18" t="str">
         <x:v>C-19</x:v>
       </x:c>
@@ -6033,7 +6033,7 @@
         <x:v>三角色服务端权限</x:v>
       </x:c>
       <x:c r="D24" s="12" t="str">
-        <x:v>guest、student/teacher、admin与越权拒绝全部通过</x:v>
+        <x:v>CAS目标明确；开发角色开关受环境变量保护，guest、student/teacher、admin与越权拒绝通过</x:v>
       </x:c>
       <x:c r="E24" s="18" t="str">
         <x:v>是非</x:v>
@@ -6071,7 +6071,7 @@
       <x:c r="AA24" s="27"/>
       <x:c r="AB24" s="27"/>
     </x:row>
-    <x:row r="25" ht="33" customHeight="1">
+    <x:row r="25" ht="24" hidden="0" customHeight="1">
       <x:c r="A25" s="18" t="str">
         <x:v>C-20</x:v>
       </x:c>
@@ -6079,10 +6079,10 @@
         <x:v>46285.625</x:v>
       </x:c>
       <x:c r="C25" s="12" t="str">
-        <x:v>Evidence-RAG三路径</x:v>
+        <x:v>带引用回答三路径</x:v>
       </x:c>
       <x:c r="D25" s="12" t="str">
-        <x:v>模型开启、关闭、证据缺失均按契约响应</x:v>
+        <x:v>模型开启、关闭、证据缺失均按契约响应；未启用Embedding</x:v>
       </x:c>
       <x:c r="E25" s="18" t="str">
         <x:v>是非</x:v>
@@ -7640,7 +7640,7 @@
       <x:c r="AA10" s="27"/>
       <x:c r="AB10" s="27"/>
     </x:row>
-    <x:row r="11">
+    <x:row r="11" ht="24" hidden="0" customHeight="1">
       <x:c r="A11" s="12" t="str">
         <x:v>H-06</x:v>
       </x:c>
@@ -7648,7 +7648,7 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="C11" s="12" t="str">
-        <x:v>HTTPS与局域网灾备演示包</x:v>
+        <x:v>React/LAN与部署清单演示包</x:v>
       </x:c>
       <x:c r="D11" s="13" t="n">
         <x:v>46285.625</x:v>
@@ -7658,10 +7658,10 @@
         <x:v>A/B</x:v>
       </x:c>
       <x:c r="G11" s="12" t="str">
-        <x:v>分别走公网和局域网关键流程</x:v>
+        <x:v>走LAN关键流程并审查云端HTTPS清单</x:v>
       </x:c>
       <x:c r="H11" s="12" t="str">
-        <x:v>健康、权限、证据、移动端、降级和恢复均通过</x:v>
+        <x:v>React前端、健康、权限、证据、移动端、降级和恢复均通过</x:v>
       </x:c>
       <x:c r="I11" s="24"/>
       <x:c r="J11" s="16"/>
@@ -13966,9 +13966,9 @@
       <x:c r="AA16" s="27"/>
       <x:c r="AB16" s="27"/>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="24" hidden="0" customHeight="1">
       <x:c r="A17" s="12" t="str">
-        <x:v>公共HTTPS与健康检查</x:v>
+        <x:v>React前端与部署检查</x:v>
       </x:c>
       <x:c r="B17" s="12" t="str">
         <x:v>C-17/C-18</x:v>
@@ -13978,7 +13978,7 @@
         <x:v>未完成</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
-        <x:v>公网URL和/healthz均需证据</x:v>
+        <x:v>React/Vite可运行，LAN健康检查和云端HTTPS清单有证据</x:v>
       </x:c>
       <x:c r="E17" s="10"/>
       <x:c r="F17" s="10"/>
@@ -14005,9 +14005,9 @@
       <x:c r="AA17" s="27"/>
       <x:c r="AB17" s="27"/>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="24" hidden="0" customHeight="1">
       <x:c r="A18" s="12" t="str">
-        <x:v>三角色权限与Evidence-RAG</x:v>
+        <x:v>三角色权限与带引用回答</x:v>
       </x:c>
       <x:c r="B18" s="12" t="str">
         <x:v>C-19/C-20</x:v>
@@ -14017,7 +14017,7 @@
         <x:v>未完成</x:v>
       </x:c>
       <x:c r="D18" s="12" t="str">
-        <x:v>服务端权限和三条检索路径</x:v>
+        <x:v>服务端权限和三条检索路径；第一周无Embedding</x:v>
       </x:c>
       <x:c r="E18" s="10"/>
       <x:c r="F18" s="10"/>

</xml_diff>

<commit_message>
fix(week1): 总览 B 角色统计范围扩至 B-17/B-18（N6:N23）
</commit_message>
<xml_diff>
--- a/docs/week1/05_本周验收台账.xlsx
+++ b/docs/week1/05_本周验收台账.xlsx
@@ -17034,15 +17034,15 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>COUNTA('B验收'!A6:A21)</f>
+        <f>COUNTA('B验收'!A6:A23)</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>COUNTIF('B验收'!N6:N21,"通过")</f>
+        <f>COUNTIF('B验收'!N6:N23,"通过")</f>
         <v/>
       </c>
       <c r="D7" s="12">
-        <f>COUNTIF('B验收'!N6:N21,"未达标")+COUNTIF('B验收'!N6:N21,"退回")</f>
+        <f>COUNTIF('B验收'!N6:N23,"未达标")+COUNTIF('B验收'!N6:N23,"退回")</f>
         <v/>
       </c>
       <c r="E7" s="12">

</xml_diff>